<commit_message>
Phase 16: motion graphics for longform (hybrid)
- AnimatedNumber.tsx: count-up primitive ($/%/×/B/M/K, commas).
- StatChart: animated growing bars, progressive line + area fill, count-up
  numbers; new modes pie / area / number (big kinetic figure). Multi-series
  CHART_COLORS.
- New 'compare' scene type (CompareCard): animated 2-column table (headings,
  center 'vs' badge, rows spring in column-by-column) + schema union +
  SceneRenderer + VerticalScene case + collectScenePhrases.
- ListCard/RecapCard: kinetic HTML rows (spring slide-in, icon chips, counting
  badges) — lists shown on screen, not narrated unseen.
- 6 money/data props: coins, dollar, bargraph, piechart, trendup, percent.
- build_manifest: SKIP_RUNTIME_GUARD=1 for sample/test renders.
- pom-sample.json proves all of it (rendered locally with Kokoro).
</commit_message>
<xml_diff>
--- a/readlark-top-100-books.xlsx
+++ b/readlark-top-100-books.xlsx
@@ -492,7 +492,7 @@
           <t>Launch Order</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="0" t="inlineStr">
         <is>
           <t>Video</t>
         </is>
@@ -569,7 +569,7 @@
       <c r="H6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="0" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
@@ -821,6 +821,11 @@
       </c>
       <c r="H13" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -4906,7 +4911,7 @@
           <t>Why this slot</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="0" t="inlineStr">
         <is>
           <t>Video</t>
         </is>
@@ -4931,7 +4936,7 @@
           <t>Anchor — flagship launch video (already live); biggest habits search term</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="0" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
@@ -4954,6 +4959,11 @@
       <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Anchor — top modern money title; broad appeal</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: clean up repo — remove pom-sample test script; xlsx video write-back
- Remove content/videos/pom-sample.json (motion-graphics test sample).
- readlark-top-100-books.xlsx: the-psychology-of-money marked produced.
- (local: cleared demo/temp artifacts in output/_samples, kokoro-samples, .build)
</commit_message>
<xml_diff>
--- a/readlark-top-100-books.xlsx
+++ b/readlark-top-100-books.xlsx
@@ -822,7 +822,7 @@
       <c r="H13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="0" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
@@ -4961,7 +4961,7 @@
           <t>Anchor — top modern money title; broad appeal</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="0" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>

</xml_diff>

<commit_message>
mark deep-work done (2026-10-18); add openpyxl to requirements
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/readlark-top-100-books.xlsx
+++ b/readlark-top-100-books.xlsx
@@ -1246,6 +1246,11 @@
       </c>
       <c r="H25" s="11" t="n">
         <v>3</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="16">
@@ -4984,6 +4989,11 @@
       <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Rankable — strong demand, lighter competition than the anchors</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
mark 7-habits done; one release bundle per book (content-<date>-<slug>) + fetch retry
Two books produced on 2026-10-18 shared the content-2026-10-18 release and the
second longform's description/thumbnail/notes overwrote the first's.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/readlark-top-100-books.xlsx
+++ b/readlark-top-100-books.xlsx
@@ -786,6 +786,11 @@
       <c r="H12" s="11" t="n">
         <v>4</v>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -1247,7 +1252,7 @@
       <c r="H25" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J25" s="0" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
@@ -4991,7 +4996,7 @@
           <t>Rankable — strong demand, lighter competition than the anchors</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="0" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
@@ -5014,6 +5019,11 @@
       <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Anchor classic — evergreen search floor</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>

</xml_diff>